<commit_message>
Add embed.py — SBERT embeddings complete, all 9 matrices serialized to interim/embeddings/
</commit_message>
<xml_diff>
--- a/input/source_data/nccer/obj/rigging/OBJ_AdvancedRigger_2E.xlsx
+++ b/input/source_data/nccer/obj/rigging/OBJ_AdvancedRigger_2E.xlsx
@@ -1042,17 +1042,84 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002C5AE0E40B4AE34D83583B8F95A6462D" ma:contentTypeVersion="0" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cf5477afdb45517565ec6d19dab827dc">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4b795196365d0a2ba85bf44c386000f7">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002C5AE0E40B4AE34D83583B8F95A6462D" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6d044a45dd115905e621c0433f4e5660">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c497ab06-58fc-49c0-91ca-a9d35bf665d3" xmlns:ns3="d264bb00-cf90-4d69-a014-b9b09b6ecdef" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="132357636063ed046e6bc674a334824d" ns2:_="" ns3:_="">
+    <xsd:import namespace="c497ab06-58fc-49c0-91ca-a9d35bf665d3"/>
+    <xsd:import namespace="d264bb00-cf90-4d69-a014-b9b09b6ecdef"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element name="documentManagement">
             <xsd:complexType>
-              <xsd:all/>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
             </xsd:complexType>
           </xsd:element>
         </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c497ab06-58fc-49c0-91ca-a9d35bf665d3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c951f097-b238-4794-a2ba-0ec37031b74f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d264bb00-cf90-4d69-a014-b9b09b6ecdef" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{0018e2c9-57cd-480a-b661-0345769eab62}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="d264bb00-cf90-4d69-a014-b9b09b6ecdef">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
@@ -1166,12 +1233,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c497ab06-58fc-49c0-91ca-a9d35bf665d3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d264bb00-cf90-4d69-a014-b9b09b6ecdef" xsi:nil="true"/>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38169AE4-2B5B-4DB7-9BD1-11994F1E4C49}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1DF3448-C489-417E-BAB4-9E9F06EFEAD1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>